<commit_message>
fix: signature lines corrected to Zenith, Opell Prima, Para (was Aliva, Opell Prima)
Updates CLAUDE.md, transform-master.js isSignature flag, search.html ranking, and rebuilds catalog.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog.generated.xlsx
+++ b/catalog.generated.xlsx
@@ -598,7 +598,7 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -651,7 +651,7 @@
         <v/>
       </c>
       <c r="M5" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -704,7 +704,7 @@
         <v/>
       </c>
       <c r="M6" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -863,7 +863,7 @@
         <v/>
       </c>
       <c r="M9" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="M10" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N10" t="str">
         <v/>
@@ -969,7 +969,7 @@
         <v/>
       </c>
       <c r="M11" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N11" t="str">
         <v/>
@@ -1022,7 +1022,7 @@
         <v/>
       </c>
       <c r="M12" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N12" t="str">
         <v/>
@@ -1075,7 +1075,7 @@
         <v/>
       </c>
       <c r="M13" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N13" t="str">
         <v/>
@@ -1128,7 +1128,7 @@
         <v/>
       </c>
       <c r="M14" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
       <c r="M15" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -1234,7 +1234,7 @@
         <v/>
       </c>
       <c r="M16" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N16" t="str">
         <v/>
@@ -1340,7 +1340,7 @@
         <v/>
       </c>
       <c r="M18" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N18" t="str">
         <v/>
@@ -1393,7 +1393,7 @@
         <v/>
       </c>
       <c r="M19" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N19" t="str">
         <v/>
@@ -1499,7 +1499,7 @@
         <v/>
       </c>
       <c r="M21" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N21" t="str">
         <v/>
@@ -1552,7 +1552,7 @@
         <v/>
       </c>
       <c r="M22" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N22" t="str">
         <v/>
@@ -1605,7 +1605,7 @@
         <v/>
       </c>
       <c r="M23" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N23" t="str">
         <v/>
@@ -1711,7 +1711,7 @@
         <v/>
       </c>
       <c r="M25" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N25" t="str">
         <v/>
@@ -1764,7 +1764,7 @@
         <v/>
       </c>
       <c r="M26" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N26" t="str">
         <v/>
@@ -1817,7 +1817,7 @@
         <v/>
       </c>
       <c r="M27" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N27" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v/>
       </c>
       <c r="M28" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="N28" t="str">
         <v/>
@@ -37571,7 +37571,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>yes</v>
+        <v/>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -37687,7 +37687,7 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>yes</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -37774,7 +37774,7 @@
         <v/>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>yes</v>
       </c>
       <c r="H13" t="str">
         <v/>

</xml_diff>